<commit_message>
[EC 02/09] Registro de Alteracoes com EC-003 e EC-004 lancadas pelo LEO — 23 registros oficiais
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="243">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -707,13 +707,65 @@
   </si>
   <si>
     <t>"pausa não vigorou no console; ver EC-002".</t>
+  </si>
+  <si>
+    <t>EC-003</t>
+  </si>
+  <si>
+    <t>EC-004</t>
+  </si>
+  <si>
+    <t>Promoção ofertas 9/9</t>
+  </si>
+  <si>
+    <t>Promoção ofertas 9/10</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">11 </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <rFont val="Carlito"/>
+      </rPr>
+      <t>SKUs: PXM 173,01 (−15%) · L2460-CP 285,33 (−15%) · L2025-T 112,97 (−15%) · L2030 101,34 (−15%) · PXP 151,10 (−10%) · L3085-B 578,02 · L3070-B 489,46 · EGC 607,16 · L2460-AML 261,15 · PG2460 223,88 · Q4070-A 947,85 (todos −10%)</t>
+    </r>
+  </si>
+  <si>
+    <t>CRIAR OFERTAS — Melhor Oferta, Clientes Prime, taxa R$ 0,00</t>
+  </si>
+  <si>
+    <t>Sem oferta</t>
+  </si>
+  <si>
+    <t>11 Melhores Ofertas programadas 07–13/09</t>
+  </si>
+  <si>
+    <t>Evento 9.9; descontos no teto da margem (medida p/ quem vendeu, Simulador piso 15% p/ o resto), cap de prudência 15%</t>
+  </si>
+  <si>
+    <t>docs/PLANO_9-9.md + Simulador Mestra v4.3.2 + Registro_Vendas</t>
+  </si>
+  <si>
+    <t>Q3060-A 499,25 (−14%) · P3060 439,82 (−14%) · P3070 554,56 (−10%) · P3050 420,90 (−10%) · P4080 963,15 (−10%)</t>
+  </si>
+  <si>
+    <t>CRIAR OFERTAS — Relâmpago, Clientes Prime, taxa R$ 0,00; dia exato definido pela Amazon (~1 semana antes)</t>
+  </si>
+  <si>
+    <t>5 Ofertas relãmpago programadas 07-13/09</t>
+  </si>
+  <si>
+    <t>Destrave de conversão (P3070 e P3050 com tráfego sem venda) + tickets do Núcleo A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -786,6 +838,12 @@
     <font>
       <u/>
       <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFF0F6FC"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -932,7 +990,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1078,6 +1136,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1532,15 +1591,15 @@
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
         <f>COUNTIF(A11:A210,"&lt;&gt;")</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B6" s="3">
         <f>COUNTIF(N11:N210,"SIM")</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O210,"SIM")</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P210,"BLOQUEADA*")</f>
@@ -1548,7 +1607,7 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
@@ -1717,7 +1776,7 @@
       </c>
       <c r="R11" s="17">
         <f t="shared" ref="R11:R42" ca="1" si="1">IF(E11="","",TODAY()-E11)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S11" s="22"/>
       <c r="T11" s="22"/>
@@ -1779,7 +1838,7 @@
       </c>
       <c r="R12" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S12" s="23"/>
       <c r="T12" s="23"/>
@@ -1839,7 +1898,7 @@
       </c>
       <c r="R13" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S13" s="23"/>
       <c r="T13" s="42"/>
@@ -1903,7 +1962,7 @@
       </c>
       <c r="R14" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S14" s="23"/>
       <c r="T14" s="23"/>
@@ -1969,7 +2028,7 @@
       </c>
       <c r="R15" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S15" s="23"/>
       <c r="T15" s="23"/>
@@ -2035,7 +2094,7 @@
       </c>
       <c r="R16" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S16" s="23"/>
       <c r="T16" s="23"/>
@@ -2101,7 +2160,7 @@
       </c>
       <c r="R17" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S17" s="23"/>
       <c r="T17" s="23"/>
@@ -2165,7 +2224,7 @@
       </c>
       <c r="R18" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S18" s="23"/>
       <c r="T18" s="23"/>
@@ -2231,7 +2290,7 @@
       </c>
       <c r="R19" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S19" s="23"/>
       <c r="T19" s="23"/>
@@ -2297,7 +2356,7 @@
       </c>
       <c r="R20" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S20" s="23"/>
       <c r="T20" s="23"/>
@@ -2361,7 +2420,7 @@
       </c>
       <c r="R21" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S21" s="23"/>
       <c r="T21" s="23"/>
@@ -2423,7 +2482,7 @@
       </c>
       <c r="R22" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S22" s="23"/>
       <c r="T22" s="23"/>
@@ -2485,7 +2544,7 @@
       </c>
       <c r="R23" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S23" s="23"/>
       <c r="T23" s="23"/>
@@ -2547,7 +2606,7 @@
       </c>
       <c r="R24" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S24" s="23"/>
       <c r="T24" s="23"/>
@@ -2613,7 +2672,7 @@
       </c>
       <c r="R25" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S25" s="23"/>
       <c r="T25" s="23"/>
@@ -2675,7 +2734,7 @@
       </c>
       <c r="R26" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S26" s="23"/>
       <c r="T26" s="23"/>
@@ -2739,7 +2798,7 @@
       </c>
       <c r="R27" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S27" s="23"/>
       <c r="T27" s="23"/>
@@ -2805,7 +2864,7 @@
       </c>
       <c r="R28" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S28" s="23"/>
       <c r="T28" s="23"/>
@@ -2871,7 +2930,7 @@
       </c>
       <c r="R29" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S29" s="23"/>
       <c r="T29" s="23"/>
@@ -2937,7 +2996,7 @@
       </c>
       <c r="R30" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S30" s="23"/>
       <c r="T30" s="23"/>
@@ -3003,7 +3062,7 @@
       </c>
       <c r="R31" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S31" s="23"/>
       <c r="T31" s="23"/>
@@ -3014,64 +3073,132 @@
         <v>227</v>
       </c>
     </row>
-    <row r="32" spans="1:22">
-      <c r="A32" s="10"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11"/>
-      <c r="O32" s="11"/>
-      <c r="P32" s="11"/>
-      <c r="Q32" s="18" t="str">
+    <row r="32" spans="1:22" ht="57">
+      <c r="A32" t="s">
+        <v>229</v>
+      </c>
+      <c r="B32" t="s">
+        <v>215</v>
+      </c>
+      <c r="C32" s="12">
+        <v>46267</v>
+      </c>
+      <c r="D32" s="12">
+        <v>46267</v>
+      </c>
+      <c r="E32" s="12">
+        <v>46267</v>
+      </c>
+      <c r="F32" s="23" t="s">
+        <v>231</v>
+      </c>
+      <c r="G32" s="51" t="s">
+        <v>233</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="I32" s="26" t="s">
+        <v>235</v>
+      </c>
+      <c r="J32" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="K32" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="L32" s="26" t="s">
+        <v>238</v>
+      </c>
+      <c r="M32" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N32" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O32" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P32" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q32" s="18">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="R32" s="19" t="str">
+        <v>46268</v>
+      </c>
+      <c r="R32" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S32" s="23"/>
       <c r="T32" s="23"/>
-      <c r="U32" s="7"/>
+      <c r="U32" s="7">
+        <v>46279</v>
+      </c>
       <c r="V32" s="28"/>
     </row>
-    <row r="33" spans="1:22">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="11"/>
-      <c r="N33" s="11"/>
-      <c r="O33" s="11"/>
-      <c r="P33" s="11"/>
-      <c r="Q33" s="18" t="str">
+    <row r="33" spans="1:22" ht="57">
+      <c r="A33" t="s">
+        <v>230</v>
+      </c>
+      <c r="B33" t="s">
+        <v>215</v>
+      </c>
+      <c r="C33" s="12">
+        <v>46267</v>
+      </c>
+      <c r="D33" s="12">
+        <v>46267</v>
+      </c>
+      <c r="E33" s="12">
+        <v>46267</v>
+      </c>
+      <c r="F33" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="G33" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="I33" s="26" t="s">
+        <v>235</v>
+      </c>
+      <c r="J33" s="26" t="s">
+        <v>241</v>
+      </c>
+      <c r="K33" s="26" t="s">
+        <v>242</v>
+      </c>
+      <c r="L33" s="26" t="s">
+        <v>238</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N33" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O33" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P33" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q33" s="18">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="R33" s="19" t="str">
+        <v>46268</v>
+      </c>
+      <c r="R33" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S33" s="23"/>
       <c r="T33" s="23"/>
-      <c r="U33" s="7"/>
+      <c r="U33" s="7">
+        <v>46279</v>
+      </c>
       <c r="V33" s="28"/>
     </row>
     <row r="34" spans="1:22">

</xml_diff>